<commit_message>
Fix a veg output bug. Before veg produce N, and main_1 and main_2 all demand N, making main_2 startve. Now veg split it in half. Still cause some problems with downstream.
</commit_message>
<xml_diff>
--- a/data/demand.xlsx
+++ b/data/demand.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="17">
   <si>
     <t xml:space="preserve">sku</t>
   </si>
@@ -43,10 +43,10 @@
     <t xml:space="preserve">fg_storage</t>
   </si>
   <si>
-    <t xml:space="preserve">sink</t>
+    <t xml:space="preserve">SKU_2</t>
   </si>
   <si>
-    <t xml:space="preserve">SKU_2</t>
+    <t xml:space="preserve">sink</t>
   </si>
   <si>
     <t xml:space="preserve">SKU_3</t>
@@ -396,30 +396,28 @@
         <v>5</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="D2" s="0"/>
       <c r="E2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>0</v>
@@ -430,13 +428,13 @@
         <v>9</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
@@ -447,13 +445,13 @@
         <v>10</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
@@ -464,13 +462,13 @@
         <v>11</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
@@ -481,13 +479,13 @@
         <v>12</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0</v>
@@ -498,13 +496,13 @@
         <v>13</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>0</v>
@@ -515,13 +513,13 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
@@ -532,13 +530,13 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
@@ -549,13 +547,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>0</v>
@@ -566,13 +564,13 @@
         <v>5</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>1440</v>
@@ -580,16 +578,16 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>1440</v>
@@ -600,13 +598,13 @@
         <v>9</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1440</v>
@@ -617,13 +615,13 @@
         <v>10</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>1440</v>
@@ -634,13 +632,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>1440</v>
@@ -651,13 +649,13 @@
         <v>12</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>1440</v>
@@ -668,13 +666,13 @@
         <v>13</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>1440</v>
@@ -685,13 +683,13 @@
         <v>14</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>1440</v>
@@ -702,13 +700,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>1440</v>
@@ -719,13 +717,13 @@
         <v>16</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>1440</v>
@@ -736,13 +734,13 @@
         <v>5</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>2880</v>
@@ -750,16 +748,16 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>2880</v>
@@ -770,13 +768,13 @@
         <v>9</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>2880</v>
@@ -787,13 +785,13 @@
         <v>10</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>2880</v>
@@ -804,13 +802,13 @@
         <v>11</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>2880</v>
@@ -821,13 +819,13 @@
         <v>12</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>2880</v>
@@ -838,13 +836,13 @@
         <v>13</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="1" t="n">
         <v>2880</v>
@@ -855,13 +853,13 @@
         <v>14</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>2880</v>
@@ -872,13 +870,13 @@
         <v>15</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>2880</v>
@@ -889,13 +887,13 @@
         <v>16</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" s="1" t="n">
         <v>2880</v>
@@ -906,13 +904,13 @@
         <v>5</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="1" t="n">
         <v>4320</v>
@@ -920,16 +918,16 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>4320</v>
@@ -940,13 +938,13 @@
         <v>9</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E34" s="1" t="n">
         <v>4320</v>
@@ -957,13 +955,13 @@
         <v>10</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E35" s="1" t="n">
         <v>4320</v>
@@ -974,13 +972,13 @@
         <v>11</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E36" s="1" t="n">
         <v>4320</v>
@@ -991,13 +989,13 @@
         <v>12</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>4320</v>
@@ -1008,13 +1006,13 @@
         <v>13</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E38" s="1" t="n">
         <v>4320</v>
@@ -1025,13 +1023,13 @@
         <v>14</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E39" s="1" t="n">
         <v>4320</v>
@@ -1042,13 +1040,13 @@
         <v>15</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>4320</v>
@@ -1059,13 +1057,13 @@
         <v>16</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E41" s="1" t="n">
         <v>4320</v>
@@ -1076,13 +1074,13 @@
         <v>5</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>5760</v>
@@ -1090,16 +1088,16 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E43" s="1" t="n">
         <v>5760</v>
@@ -1110,13 +1108,13 @@
         <v>9</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E44" s="1" t="n">
         <v>5760</v>
@@ -1127,13 +1125,13 @@
         <v>10</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E45" s="1" t="n">
         <v>5760</v>
@@ -1144,13 +1142,13 @@
         <v>11</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>5760</v>
@@ -1161,13 +1159,13 @@
         <v>12</v>
       </c>
       <c r="B47" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E47" s="1" t="n">
         <v>5760</v>
@@ -1178,13 +1176,13 @@
         <v>13</v>
       </c>
       <c r="B48" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E48" s="1" t="n">
         <v>5760</v>
@@ -1195,13 +1193,13 @@
         <v>14</v>
       </c>
       <c r="B49" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E49" s="1" t="n">
         <v>5760</v>
@@ -1212,13 +1210,13 @@
         <v>15</v>
       </c>
       <c r="B50" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E50" s="1" t="n">
         <v>5760</v>
@@ -1229,13 +1227,13 @@
         <v>16</v>
       </c>
       <c r="B51" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E51" s="1" t="n">
         <v>5760</v>
@@ -1246,13 +1244,13 @@
         <v>5</v>
       </c>
       <c r="B52" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E52" s="1" t="n">
         <v>7200</v>
@@ -1260,16 +1258,16 @@
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B53" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E53" s="1" t="n">
         <v>7200</v>
@@ -1280,13 +1278,13 @@
         <v>9</v>
       </c>
       <c r="B54" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E54" s="1" t="n">
         <v>7200</v>
@@ -1297,13 +1295,13 @@
         <v>10</v>
       </c>
       <c r="B55" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E55" s="1" t="n">
         <v>7200</v>
@@ -1314,13 +1312,13 @@
         <v>11</v>
       </c>
       <c r="B56" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>7200</v>
@@ -1331,13 +1329,13 @@
         <v>12</v>
       </c>
       <c r="B57" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>7200</v>
@@ -1348,13 +1346,13 @@
         <v>13</v>
       </c>
       <c r="B58" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>7200</v>
@@ -1365,13 +1363,13 @@
         <v>14</v>
       </c>
       <c r="B59" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E59" s="1" t="n">
         <v>7200</v>
@@ -1382,13 +1380,13 @@
         <v>15</v>
       </c>
       <c r="B60" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E60" s="1" t="n">
         <v>7200</v>
@@ -1399,13 +1397,13 @@
         <v>16</v>
       </c>
       <c r="B61" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>7200</v>
@@ -1416,13 +1414,13 @@
         <v>5</v>
       </c>
       <c r="B62" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>8640</v>
@@ -1430,16 +1428,16 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B63" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E63" s="1" t="n">
         <v>8640</v>
@@ -1450,13 +1448,13 @@
         <v>9</v>
       </c>
       <c r="B64" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>8640</v>
@@ -1467,13 +1465,13 @@
         <v>10</v>
       </c>
       <c r="B65" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>8640</v>
@@ -1484,13 +1482,13 @@
         <v>11</v>
       </c>
       <c r="B66" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>8640</v>
@@ -1501,13 +1499,13 @@
         <v>12</v>
       </c>
       <c r="B67" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>8640</v>
@@ -1518,13 +1516,13 @@
         <v>13</v>
       </c>
       <c r="B68" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E68" s="1" t="n">
         <v>8640</v>
@@ -1535,13 +1533,13 @@
         <v>14</v>
       </c>
       <c r="B69" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E69" s="1" t="n">
         <v>8640</v>
@@ -1552,13 +1550,13 @@
         <v>15</v>
       </c>
       <c r="B70" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>8640</v>
@@ -1569,13 +1567,13 @@
         <v>16</v>
       </c>
       <c r="B71" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E71" s="1" t="n">
         <v>8640</v>
@@ -1586,13 +1584,13 @@
         <v>5</v>
       </c>
       <c r="B72" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E72" s="1" t="n">
         <v>10080</v>
@@ -1600,16 +1598,16 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B73" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>10080</v>
@@ -1620,13 +1618,13 @@
         <v>9</v>
       </c>
       <c r="B74" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E74" s="1" t="n">
         <v>10080</v>
@@ -1637,13 +1635,13 @@
         <v>10</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E75" s="1" t="n">
         <v>10080</v>
@@ -1654,13 +1652,13 @@
         <v>11</v>
       </c>
       <c r="B76" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E76" s="1" t="n">
         <v>10080</v>
@@ -1671,13 +1669,13 @@
         <v>12</v>
       </c>
       <c r="B77" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E77" s="1" t="n">
         <v>10080</v>
@@ -1688,13 +1686,13 @@
         <v>13</v>
       </c>
       <c r="B78" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E78" s="1" t="n">
         <v>10080</v>
@@ -1705,13 +1703,13 @@
         <v>14</v>
       </c>
       <c r="B79" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E79" s="1" t="n">
         <v>10080</v>
@@ -1722,13 +1720,13 @@
         <v>15</v>
       </c>
       <c r="B80" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E80" s="1" t="n">
         <v>10080</v>
@@ -1739,13 +1737,13 @@
         <v>16</v>
       </c>
       <c r="B81" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E81" s="1" t="n">
         <v>10080</v>
@@ -1756,13 +1754,13 @@
         <v>5</v>
       </c>
       <c r="B82" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E82" s="1" t="n">
         <v>11520</v>
@@ -1770,16 +1768,16 @@
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B83" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E83" s="1" t="n">
         <v>11520</v>
@@ -1790,13 +1788,13 @@
         <v>9</v>
       </c>
       <c r="B84" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E84" s="1" t="n">
         <v>11520</v>
@@ -1807,13 +1805,13 @@
         <v>10</v>
       </c>
       <c r="B85" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E85" s="1" t="n">
         <v>11520</v>
@@ -1824,13 +1822,13 @@
         <v>11</v>
       </c>
       <c r="B86" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E86" s="1" t="n">
         <v>11520</v>
@@ -1841,13 +1839,13 @@
         <v>12</v>
       </c>
       <c r="B87" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E87" s="1" t="n">
         <v>11520</v>
@@ -1858,13 +1856,13 @@
         <v>13</v>
       </c>
       <c r="B88" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E88" s="1" t="n">
         <v>11520</v>
@@ -1875,13 +1873,13 @@
         <v>14</v>
       </c>
       <c r="B89" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E89" s="1" t="n">
         <v>11520</v>
@@ -1892,13 +1890,13 @@
         <v>15</v>
       </c>
       <c r="B90" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E90" s="1" t="n">
         <v>11520</v>
@@ -1909,13 +1907,13 @@
         <v>16</v>
       </c>
       <c r="B91" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E91" s="1" t="n">
         <v>11520</v>
@@ -1926,13 +1924,13 @@
         <v>5</v>
       </c>
       <c r="B92" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E92" s="1" t="n">
         <v>12960</v>
@@ -1940,16 +1938,16 @@
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B93" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E93" s="1" t="n">
         <v>12960</v>
@@ -1960,13 +1958,13 @@
         <v>9</v>
       </c>
       <c r="B94" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E94" s="1" t="n">
         <v>12960</v>
@@ -1977,13 +1975,13 @@
         <v>10</v>
       </c>
       <c r="B95" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E95" s="1" t="n">
         <v>12960</v>
@@ -1994,13 +1992,13 @@
         <v>11</v>
       </c>
       <c r="B96" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E96" s="1" t="n">
         <v>12960</v>
@@ -2011,13 +2009,13 @@
         <v>12</v>
       </c>
       <c r="B97" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E97" s="1" t="n">
         <v>12960</v>
@@ -2028,13 +2026,13 @@
         <v>13</v>
       </c>
       <c r="B98" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E98" s="1" t="n">
         <v>12960</v>
@@ -2045,13 +2043,13 @@
         <v>14</v>
       </c>
       <c r="B99" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E99" s="1" t="n">
         <v>12960</v>
@@ -2062,13 +2060,13 @@
         <v>15</v>
       </c>
       <c r="B100" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E100" s="1" t="n">
         <v>12960</v>
@@ -2079,13 +2077,13 @@
         <v>16</v>
       </c>
       <c r="B101" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E101" s="1" t="n">
         <v>12960</v>
@@ -2096,13 +2094,13 @@
         <v>5</v>
       </c>
       <c r="B102" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E102" s="1" t="n">
         <v>14400</v>
@@ -2110,16 +2108,16 @@
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B103" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E103" s="1" t="n">
         <v>14400</v>
@@ -2130,13 +2128,13 @@
         <v>9</v>
       </c>
       <c r="B104" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E104" s="1" t="n">
         <v>14400</v>
@@ -2147,13 +2145,13 @@
         <v>10</v>
       </c>
       <c r="B105" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E105" s="1" t="n">
         <v>14400</v>
@@ -2164,13 +2162,13 @@
         <v>11</v>
       </c>
       <c r="B106" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E106" s="1" t="n">
         <v>14400</v>
@@ -2181,13 +2179,13 @@
         <v>12</v>
       </c>
       <c r="B107" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E107" s="1" t="n">
         <v>14400</v>
@@ -2198,13 +2196,13 @@
         <v>13</v>
       </c>
       <c r="B108" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E108" s="1" t="n">
         <v>14400</v>
@@ -2215,13 +2213,13 @@
         <v>14</v>
       </c>
       <c r="B109" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E109" s="1" t="n">
         <v>14400</v>
@@ -2232,13 +2230,13 @@
         <v>15</v>
       </c>
       <c r="B110" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E110" s="1" t="n">
         <v>14400</v>
@@ -2249,13 +2247,13 @@
         <v>16</v>
       </c>
       <c r="B111" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E111" s="1" t="n">
         <v>14400</v>
@@ -2266,13 +2264,13 @@
         <v>5</v>
       </c>
       <c r="B112" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E112" s="1" t="n">
         <v>15840</v>
@@ -2280,16 +2278,16 @@
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B113" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E113" s="1" t="n">
         <v>15840</v>
@@ -2300,13 +2298,13 @@
         <v>9</v>
       </c>
       <c r="B114" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E114" s="1" t="n">
         <v>15840</v>
@@ -2317,13 +2315,13 @@
         <v>10</v>
       </c>
       <c r="B115" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E115" s="1" t="n">
         <v>15840</v>
@@ -2334,13 +2332,13 @@
         <v>11</v>
       </c>
       <c r="B116" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E116" s="1" t="n">
         <v>15840</v>
@@ -2351,13 +2349,13 @@
         <v>12</v>
       </c>
       <c r="B117" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E117" s="1" t="n">
         <v>15840</v>
@@ -2368,13 +2366,13 @@
         <v>13</v>
       </c>
       <c r="B118" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E118" s="1" t="n">
         <v>15840</v>
@@ -2385,13 +2383,13 @@
         <v>14</v>
       </c>
       <c r="B119" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E119" s="1" t="n">
         <v>15840</v>
@@ -2402,13 +2400,13 @@
         <v>15</v>
       </c>
       <c r="B120" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E120" s="1" t="n">
         <v>15840</v>
@@ -2419,13 +2417,13 @@
         <v>16</v>
       </c>
       <c r="B121" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E121" s="1" t="n">
         <v>15840</v>
@@ -2436,13 +2434,13 @@
         <v>5</v>
       </c>
       <c r="B122" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E122" s="1" t="n">
         <v>17280</v>
@@ -2450,16 +2448,16 @@
     </row>
     <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B123" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E123" s="1" t="n">
         <v>17280</v>
@@ -2470,13 +2468,13 @@
         <v>9</v>
       </c>
       <c r="B124" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E124" s="1" t="n">
         <v>17280</v>
@@ -2487,13 +2485,13 @@
         <v>10</v>
       </c>
       <c r="B125" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E125" s="1" t="n">
         <v>17280</v>
@@ -2504,13 +2502,13 @@
         <v>11</v>
       </c>
       <c r="B126" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E126" s="1" t="n">
         <v>17280</v>
@@ -2521,13 +2519,13 @@
         <v>12</v>
       </c>
       <c r="B127" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E127" s="1" t="n">
         <v>17280</v>
@@ -2538,13 +2536,13 @@
         <v>13</v>
       </c>
       <c r="B128" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E128" s="1" t="n">
         <v>17280</v>
@@ -2555,13 +2553,13 @@
         <v>14</v>
       </c>
       <c r="B129" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E129" s="1" t="n">
         <v>17280</v>
@@ -2572,13 +2570,13 @@
         <v>15</v>
       </c>
       <c r="B130" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E130" s="1" t="n">
         <v>17280</v>
@@ -2589,13 +2587,13 @@
         <v>16</v>
       </c>
       <c r="B131" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E131" s="1" t="n">
         <v>17280</v>
@@ -2606,13 +2604,13 @@
         <v>5</v>
       </c>
       <c r="B132" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E132" s="1" t="n">
         <v>18720</v>
@@ -2620,16 +2618,16 @@
     </row>
     <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B133" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E133" s="1" t="n">
         <v>18720</v>
@@ -2640,13 +2638,13 @@
         <v>9</v>
       </c>
       <c r="B134" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E134" s="1" t="n">
         <v>18720</v>
@@ -2657,13 +2655,13 @@
         <v>10</v>
       </c>
       <c r="B135" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E135" s="1" t="n">
         <v>18720</v>
@@ -2674,13 +2672,13 @@
         <v>11</v>
       </c>
       <c r="B136" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E136" s="1" t="n">
         <v>18720</v>
@@ -2691,13 +2689,13 @@
         <v>12</v>
       </c>
       <c r="B137" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E137" s="1" t="n">
         <v>18720</v>
@@ -2708,13 +2706,13 @@
         <v>13</v>
       </c>
       <c r="B138" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E138" s="1" t="n">
         <v>18720</v>
@@ -2725,13 +2723,13 @@
         <v>14</v>
       </c>
       <c r="B139" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E139" s="1" t="n">
         <v>18720</v>
@@ -2742,13 +2740,13 @@
         <v>15</v>
       </c>
       <c r="B140" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D140" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E140" s="1" t="n">
         <v>18720</v>
@@ -2759,13 +2757,13 @@
         <v>16</v>
       </c>
       <c r="B141" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E141" s="1" t="n">
         <v>18720</v>
@@ -2776,13 +2774,13 @@
         <v>5</v>
       </c>
       <c r="B142" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E142" s="1" t="n">
         <v>20160</v>
@@ -2790,16 +2788,16 @@
     </row>
     <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B143" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E143" s="1" t="n">
         <v>20160</v>
@@ -2810,13 +2808,13 @@
         <v>9</v>
       </c>
       <c r="B144" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E144" s="1" t="n">
         <v>20160</v>
@@ -2827,13 +2825,13 @@
         <v>10</v>
       </c>
       <c r="B145" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E145" s="1" t="n">
         <v>20160</v>
@@ -2844,13 +2842,13 @@
         <v>11</v>
       </c>
       <c r="B146" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E146" s="1" t="n">
         <v>20160</v>
@@ -2861,13 +2859,13 @@
         <v>12</v>
       </c>
       <c r="B147" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E147" s="1" t="n">
         <v>20160</v>
@@ -2878,13 +2876,13 @@
         <v>13</v>
       </c>
       <c r="B148" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E148" s="1" t="n">
         <v>20160</v>
@@ -2895,13 +2893,13 @@
         <v>14</v>
       </c>
       <c r="B149" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E149" s="1" t="n">
         <v>20160</v>
@@ -2912,13 +2910,13 @@
         <v>15</v>
       </c>
       <c r="B150" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E150" s="1" t="n">
         <v>20160</v>
@@ -2929,13 +2927,13 @@
         <v>16</v>
       </c>
       <c r="B151" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E151" s="1" t="n">
         <v>20160</v>
@@ -2946,13 +2944,13 @@
         <v>5</v>
       </c>
       <c r="B152" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E152" s="1" t="n">
         <v>21600</v>
@@ -2960,16 +2958,16 @@
     </row>
     <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B153" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E153" s="1" t="n">
         <v>21600</v>
@@ -2980,13 +2978,13 @@
         <v>9</v>
       </c>
       <c r="B154" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E154" s="1" t="n">
         <v>21600</v>
@@ -2997,13 +2995,13 @@
         <v>10</v>
       </c>
       <c r="B155" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E155" s="1" t="n">
         <v>21600</v>
@@ -3014,13 +3012,13 @@
         <v>11</v>
       </c>
       <c r="B156" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E156" s="1" t="n">
         <v>21600</v>
@@ -3031,13 +3029,13 @@
         <v>12</v>
       </c>
       <c r="B157" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E157" s="1" t="n">
         <v>21600</v>
@@ -3048,13 +3046,13 @@
         <v>13</v>
       </c>
       <c r="B158" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E158" s="1" t="n">
         <v>21600</v>
@@ -3065,13 +3063,13 @@
         <v>14</v>
       </c>
       <c r="B159" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E159" s="1" t="n">
         <v>21600</v>
@@ -3082,13 +3080,13 @@
         <v>15</v>
       </c>
       <c r="B160" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E160" s="1" t="n">
         <v>21600</v>
@@ -3099,13 +3097,13 @@
         <v>16</v>
       </c>
       <c r="B161" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E161" s="1" t="n">
         <v>21600</v>
@@ -3116,13 +3114,13 @@
         <v>5</v>
       </c>
       <c r="B162" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E162" s="1" t="n">
         <v>23040</v>
@@ -3130,16 +3128,16 @@
     </row>
     <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B163" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E163" s="1" t="n">
         <v>23040</v>
@@ -3150,13 +3148,13 @@
         <v>9</v>
       </c>
       <c r="B164" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E164" s="1" t="n">
         <v>23040</v>
@@ -3167,13 +3165,13 @@
         <v>10</v>
       </c>
       <c r="B165" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E165" s="1" t="n">
         <v>23040</v>
@@ -3184,13 +3182,13 @@
         <v>11</v>
       </c>
       <c r="B166" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E166" s="1" t="n">
         <v>23040</v>
@@ -3201,13 +3199,13 @@
         <v>12</v>
       </c>
       <c r="B167" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D167" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E167" s="1" t="n">
         <v>23040</v>
@@ -3218,13 +3216,13 @@
         <v>13</v>
       </c>
       <c r="B168" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D168" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E168" s="1" t="n">
         <v>23040</v>
@@ -3235,13 +3233,13 @@
         <v>14</v>
       </c>
       <c r="B169" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D169" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E169" s="1" t="n">
         <v>23040</v>
@@ -3252,13 +3250,13 @@
         <v>15</v>
       </c>
       <c r="B170" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D170" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E170" s="1" t="n">
         <v>23040</v>
@@ -3269,13 +3267,13 @@
         <v>16</v>
       </c>
       <c r="B171" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D171" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E171" s="1" t="n">
         <v>23040</v>
@@ -3286,13 +3284,13 @@
         <v>5</v>
       </c>
       <c r="B172" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D172" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E172" s="1" t="n">
         <v>24480</v>
@@ -3300,16 +3298,16 @@
     </row>
     <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B173" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D173" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E173" s="1" t="n">
         <v>24480</v>
@@ -3320,13 +3318,13 @@
         <v>9</v>
       </c>
       <c r="B174" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E174" s="1" t="n">
         <v>24480</v>
@@ -3337,13 +3335,13 @@
         <v>10</v>
       </c>
       <c r="B175" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E175" s="1" t="n">
         <v>24480</v>
@@ -3354,13 +3352,13 @@
         <v>11</v>
       </c>
       <c r="B176" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D176" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E176" s="1" t="n">
         <v>24480</v>
@@ -3371,13 +3369,13 @@
         <v>12</v>
       </c>
       <c r="B177" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D177" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E177" s="1" t="n">
         <v>24480</v>
@@ -3388,13 +3386,13 @@
         <v>13</v>
       </c>
       <c r="B178" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D178" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E178" s="1" t="n">
         <v>24480</v>
@@ -3405,13 +3403,13 @@
         <v>14</v>
       </c>
       <c r="B179" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E179" s="1" t="n">
         <v>24480</v>
@@ -3422,13 +3420,13 @@
         <v>15</v>
       </c>
       <c r="B180" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D180" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E180" s="1" t="n">
         <v>24480</v>
@@ -3439,13 +3437,13 @@
         <v>16</v>
       </c>
       <c r="B181" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D181" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E181" s="1" t="n">
         <v>24480</v>
@@ -3456,13 +3454,13 @@
         <v>5</v>
       </c>
       <c r="B182" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D182" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E182" s="1" t="n">
         <v>25920</v>
@@ -3470,16 +3468,16 @@
     </row>
     <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B183" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D183" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E183" s="1" t="n">
         <v>25920</v>
@@ -3490,13 +3488,13 @@
         <v>9</v>
       </c>
       <c r="B184" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D184" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E184" s="1" t="n">
         <v>25920</v>
@@ -3507,13 +3505,13 @@
         <v>10</v>
       </c>
       <c r="B185" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D185" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E185" s="1" t="n">
         <v>25920</v>
@@ -3524,13 +3522,13 @@
         <v>11</v>
       </c>
       <c r="B186" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D186" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E186" s="1" t="n">
         <v>25920</v>
@@ -3541,13 +3539,13 @@
         <v>12</v>
       </c>
       <c r="B187" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D187" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E187" s="1" t="n">
         <v>25920</v>
@@ -3558,13 +3556,13 @@
         <v>13</v>
       </c>
       <c r="B188" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D188" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E188" s="1" t="n">
         <v>25920</v>
@@ -3575,13 +3573,13 @@
         <v>14</v>
       </c>
       <c r="B189" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D189" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E189" s="1" t="n">
         <v>25920</v>
@@ -3592,13 +3590,13 @@
         <v>15</v>
       </c>
       <c r="B190" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C190" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D190" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E190" s="1" t="n">
         <v>25920</v>
@@ -3609,13 +3607,13 @@
         <v>16</v>
       </c>
       <c r="B191" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C191" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D191" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E191" s="1" t="n">
         <v>25920</v>
@@ -3626,13 +3624,13 @@
         <v>5</v>
       </c>
       <c r="B192" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D192" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E192" s="1" t="n">
         <v>27360</v>
@@ -3640,16 +3638,16 @@
     </row>
     <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B193" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D193" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E193" s="1" t="n">
         <v>27360</v>
@@ -3660,13 +3658,13 @@
         <v>9</v>
       </c>
       <c r="B194" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C194" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D194" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E194" s="1" t="n">
         <v>27360</v>
@@ -3677,13 +3675,13 @@
         <v>10</v>
       </c>
       <c r="B195" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D195" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E195" s="1" t="n">
         <v>27360</v>
@@ -3694,13 +3692,13 @@
         <v>11</v>
       </c>
       <c r="B196" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D196" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E196" s="1" t="n">
         <v>27360</v>
@@ -3711,13 +3709,13 @@
         <v>12</v>
       </c>
       <c r="B197" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D197" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E197" s="1" t="n">
         <v>27360</v>
@@ -3728,13 +3726,13 @@
         <v>13</v>
       </c>
       <c r="B198" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D198" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E198" s="1" t="n">
         <v>27360</v>
@@ -3745,13 +3743,13 @@
         <v>14</v>
       </c>
       <c r="B199" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D199" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E199" s="1" t="n">
         <v>27360</v>
@@ -3762,13 +3760,13 @@
         <v>15</v>
       </c>
       <c r="B200" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C200" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D200" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E200" s="1" t="n">
         <v>27360</v>
@@ -3779,13 +3777,13 @@
         <v>16</v>
       </c>
       <c r="B201" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C201" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D201" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E201" s="1" t="n">
         <v>27360</v>
@@ -3796,13 +3794,13 @@
         <v>5</v>
       </c>
       <c r="B202" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C202" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D202" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E202" s="1" t="n">
         <v>28800</v>
@@ -3810,16 +3808,16 @@
     </row>
     <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B203" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C203" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D203" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E203" s="1" t="n">
         <v>28800</v>
@@ -3830,13 +3828,13 @@
         <v>9</v>
       </c>
       <c r="B204" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C204" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D204" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E204" s="1" t="n">
         <v>28800</v>
@@ -3847,13 +3845,13 @@
         <v>10</v>
       </c>
       <c r="B205" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C205" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D205" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E205" s="1" t="n">
         <v>28800</v>
@@ -3864,13 +3862,13 @@
         <v>11</v>
       </c>
       <c r="B206" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C206" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D206" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E206" s="1" t="n">
         <v>28800</v>
@@ -3881,13 +3879,13 @@
         <v>12</v>
       </c>
       <c r="B207" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C207" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D207" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E207" s="1" t="n">
         <v>28800</v>
@@ -3898,13 +3896,13 @@
         <v>13</v>
       </c>
       <c r="B208" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C208" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D208" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E208" s="1" t="n">
         <v>28800</v>
@@ -3915,13 +3913,13 @@
         <v>14</v>
       </c>
       <c r="B209" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C209" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D209" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E209" s="1" t="n">
         <v>28800</v>
@@ -3932,13 +3930,13 @@
         <v>15</v>
       </c>
       <c r="B210" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C210" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D210" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E210" s="1" t="n">
         <v>28800</v>
@@ -3949,13 +3947,13 @@
         <v>16</v>
       </c>
       <c r="B211" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C211" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D211" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E211" s="1" t="n">
         <v>28800</v>
@@ -3966,13 +3964,13 @@
         <v>5</v>
       </c>
       <c r="B212" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C212" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D212" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E212" s="1" t="n">
         <v>30240</v>
@@ -3980,16 +3978,16 @@
     </row>
     <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B213" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C213" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D213" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E213" s="1" t="n">
         <v>30240</v>
@@ -4000,13 +3998,13 @@
         <v>9</v>
       </c>
       <c r="B214" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C214" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D214" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E214" s="1" t="n">
         <v>30240</v>
@@ -4017,13 +4015,13 @@
         <v>10</v>
       </c>
       <c r="B215" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C215" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D215" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E215" s="1" t="n">
         <v>30240</v>
@@ -4034,13 +4032,13 @@
         <v>11</v>
       </c>
       <c r="B216" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C216" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D216" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E216" s="1" t="n">
         <v>30240</v>
@@ -4051,13 +4049,13 @@
         <v>12</v>
       </c>
       <c r="B217" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C217" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D217" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E217" s="1" t="n">
         <v>30240</v>
@@ -4068,13 +4066,13 @@
         <v>13</v>
       </c>
       <c r="B218" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C218" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D218" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E218" s="1" t="n">
         <v>30240</v>
@@ -4085,13 +4083,13 @@
         <v>14</v>
       </c>
       <c r="B219" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C219" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D219" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E219" s="1" t="n">
         <v>30240</v>
@@ -4102,13 +4100,13 @@
         <v>15</v>
       </c>
       <c r="B220" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C220" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D220" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E220" s="1" t="n">
         <v>30240</v>
@@ -4119,13 +4117,13 @@
         <v>16</v>
       </c>
       <c r="B221" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C221" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D221" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E221" s="1" t="n">
         <v>30240</v>
@@ -4136,13 +4134,13 @@
         <v>5</v>
       </c>
       <c r="B222" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C222" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D222" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E222" s="1" t="n">
         <v>31680</v>
@@ -4150,16 +4148,16 @@
     </row>
     <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B223" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C223" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D223" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E223" s="1" t="n">
         <v>31680</v>
@@ -4170,13 +4168,13 @@
         <v>9</v>
       </c>
       <c r="B224" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C224" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D224" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E224" s="1" t="n">
         <v>31680</v>
@@ -4187,13 +4185,13 @@
         <v>10</v>
       </c>
       <c r="B225" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C225" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D225" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E225" s="1" t="n">
         <v>31680</v>
@@ -4204,13 +4202,13 @@
         <v>11</v>
       </c>
       <c r="B226" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C226" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D226" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E226" s="1" t="n">
         <v>31680</v>
@@ -4221,13 +4219,13 @@
         <v>12</v>
       </c>
       <c r="B227" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C227" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D227" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E227" s="1" t="n">
         <v>31680</v>
@@ -4238,13 +4236,13 @@
         <v>13</v>
       </c>
       <c r="B228" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C228" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D228" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E228" s="1" t="n">
         <v>31680</v>
@@ -4255,13 +4253,13 @@
         <v>14</v>
       </c>
       <c r="B229" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C229" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D229" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E229" s="1" t="n">
         <v>31680</v>
@@ -4272,13 +4270,13 @@
         <v>15</v>
       </c>
       <c r="B230" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C230" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D230" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E230" s="1" t="n">
         <v>31680</v>
@@ -4289,13 +4287,13 @@
         <v>16</v>
       </c>
       <c r="B231" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C231" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D231" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E231" s="1" t="n">
         <v>31680</v>
@@ -4306,13 +4304,13 @@
         <v>5</v>
       </c>
       <c r="B232" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C232" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D232" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E232" s="1" t="n">
         <v>33120</v>
@@ -4320,16 +4318,16 @@
     </row>
     <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B233" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C233" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D233" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E233" s="1" t="n">
         <v>33120</v>
@@ -4340,13 +4338,13 @@
         <v>9</v>
       </c>
       <c r="B234" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C234" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D234" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E234" s="1" t="n">
         <v>33120</v>
@@ -4357,13 +4355,13 @@
         <v>10</v>
       </c>
       <c r="B235" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C235" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D235" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E235" s="1" t="n">
         <v>33120</v>
@@ -4374,13 +4372,13 @@
         <v>11</v>
       </c>
       <c r="B236" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D236" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E236" s="1" t="n">
         <v>33120</v>
@@ -4391,13 +4389,13 @@
         <v>12</v>
       </c>
       <c r="B237" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C237" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D237" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E237" s="1" t="n">
         <v>33120</v>
@@ -4408,13 +4406,13 @@
         <v>13</v>
       </c>
       <c r="B238" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C238" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D238" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E238" s="1" t="n">
         <v>33120</v>
@@ -4425,13 +4423,13 @@
         <v>14</v>
       </c>
       <c r="B239" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C239" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D239" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E239" s="1" t="n">
         <v>33120</v>
@@ -4442,13 +4440,13 @@
         <v>15</v>
       </c>
       <c r="B240" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C240" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D240" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E240" s="1" t="n">
         <v>33120</v>
@@ -4459,13 +4457,13 @@
         <v>16</v>
       </c>
       <c r="B241" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C241" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D241" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E241" s="1" t="n">
         <v>33120</v>
@@ -4476,13 +4474,13 @@
         <v>5</v>
       </c>
       <c r="B242" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C242" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D242" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E242" s="1" t="n">
         <v>34560</v>
@@ -4490,16 +4488,16 @@
     </row>
     <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B243" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C243" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D243" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E243" s="1" t="n">
         <v>34560</v>
@@ -4510,13 +4508,13 @@
         <v>9</v>
       </c>
       <c r="B244" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C244" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D244" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E244" s="1" t="n">
         <v>34560</v>
@@ -4527,13 +4525,13 @@
         <v>10</v>
       </c>
       <c r="B245" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C245" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D245" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E245" s="1" t="n">
         <v>34560</v>
@@ -4544,13 +4542,13 @@
         <v>11</v>
       </c>
       <c r="B246" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C246" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D246" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E246" s="1" t="n">
         <v>34560</v>
@@ -4561,13 +4559,13 @@
         <v>12</v>
       </c>
       <c r="B247" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C247" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D247" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E247" s="1" t="n">
         <v>34560</v>
@@ -4578,13 +4576,13 @@
         <v>13</v>
       </c>
       <c r="B248" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C248" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D248" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E248" s="1" t="n">
         <v>34560</v>
@@ -4595,13 +4593,13 @@
         <v>14</v>
       </c>
       <c r="B249" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C249" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D249" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E249" s="1" t="n">
         <v>34560</v>
@@ -4612,13 +4610,13 @@
         <v>15</v>
       </c>
       <c r="B250" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C250" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D250" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E250" s="1" t="n">
         <v>34560</v>
@@ -4629,13 +4627,13 @@
         <v>16</v>
       </c>
       <c r="B251" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C251" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D251" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E251" s="1" t="n">
         <v>34560</v>
@@ -4646,13 +4644,13 @@
         <v>5</v>
       </c>
       <c r="B252" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C252" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D252" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E252" s="1" t="n">
         <v>36000</v>
@@ -4660,16 +4658,16 @@
     </row>
     <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B253" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C253" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D253" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E253" s="1" t="n">
         <v>36000</v>
@@ -4680,13 +4678,13 @@
         <v>9</v>
       </c>
       <c r="B254" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C254" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D254" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E254" s="1" t="n">
         <v>36000</v>
@@ -4697,13 +4695,13 @@
         <v>10</v>
       </c>
       <c r="B255" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C255" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D255" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E255" s="1" t="n">
         <v>36000</v>
@@ -4714,13 +4712,13 @@
         <v>11</v>
       </c>
       <c r="B256" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C256" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D256" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E256" s="1" t="n">
         <v>36000</v>
@@ -4731,13 +4729,13 @@
         <v>12</v>
       </c>
       <c r="B257" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C257" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D257" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E257" s="1" t="n">
         <v>36000</v>
@@ -4748,13 +4746,13 @@
         <v>13</v>
       </c>
       <c r="B258" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C258" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D258" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E258" s="1" t="n">
         <v>36000</v>
@@ -4765,13 +4763,13 @@
         <v>14</v>
       </c>
       <c r="B259" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C259" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D259" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E259" s="1" t="n">
         <v>36000</v>
@@ -4782,13 +4780,13 @@
         <v>15</v>
       </c>
       <c r="B260" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C260" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D260" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E260" s="1" t="n">
         <v>36000</v>
@@ -4799,13 +4797,13 @@
         <v>16</v>
       </c>
       <c r="B261" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C261" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D261" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E261" s="1" t="n">
         <v>36000</v>
@@ -4816,13 +4814,13 @@
         <v>5</v>
       </c>
       <c r="B262" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C262" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D262" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E262" s="1" t="n">
         <v>37440</v>
@@ -4830,16 +4828,16 @@
     </row>
     <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B263" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C263" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D263" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E263" s="1" t="n">
         <v>37440</v>
@@ -4850,13 +4848,13 @@
         <v>9</v>
       </c>
       <c r="B264" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C264" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D264" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E264" s="1" t="n">
         <v>37440</v>
@@ -4867,13 +4865,13 @@
         <v>10</v>
       </c>
       <c r="B265" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C265" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D265" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E265" s="1" t="n">
         <v>37440</v>
@@ -4884,13 +4882,13 @@
         <v>11</v>
       </c>
       <c r="B266" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C266" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D266" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E266" s="1" t="n">
         <v>37440</v>
@@ -4901,13 +4899,13 @@
         <v>12</v>
       </c>
       <c r="B267" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C267" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D267" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E267" s="1" t="n">
         <v>37440</v>
@@ -4918,13 +4916,13 @@
         <v>13</v>
       </c>
       <c r="B268" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C268" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D268" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E268" s="1" t="n">
         <v>37440</v>
@@ -4935,13 +4933,13 @@
         <v>14</v>
       </c>
       <c r="B269" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C269" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D269" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E269" s="1" t="n">
         <v>37440</v>
@@ -4952,13 +4950,13 @@
         <v>15</v>
       </c>
       <c r="B270" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C270" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D270" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E270" s="1" t="n">
         <v>37440</v>
@@ -4969,13 +4967,13 @@
         <v>16</v>
       </c>
       <c r="B271" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C271" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D271" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E271" s="1" t="n">
         <v>37440</v>
@@ -4986,13 +4984,13 @@
         <v>5</v>
       </c>
       <c r="B272" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C272" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D272" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E272" s="1" t="n">
         <v>38880</v>
@@ -5000,16 +4998,16 @@
     </row>
     <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B273" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C273" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D273" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E273" s="1" t="n">
         <v>38880</v>
@@ -5020,13 +5018,13 @@
         <v>9</v>
       </c>
       <c r="B274" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C274" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D274" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E274" s="1" t="n">
         <v>38880</v>
@@ -5037,13 +5035,13 @@
         <v>10</v>
       </c>
       <c r="B275" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C275" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D275" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E275" s="1" t="n">
         <v>38880</v>
@@ -5054,13 +5052,13 @@
         <v>11</v>
       </c>
       <c r="B276" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C276" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D276" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E276" s="1" t="n">
         <v>38880</v>
@@ -5071,13 +5069,13 @@
         <v>12</v>
       </c>
       <c r="B277" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C277" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D277" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E277" s="1" t="n">
         <v>38880</v>
@@ -5088,13 +5086,13 @@
         <v>13</v>
       </c>
       <c r="B278" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C278" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D278" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E278" s="1" t="n">
         <v>38880</v>
@@ -5105,13 +5103,13 @@
         <v>14</v>
       </c>
       <c r="B279" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C279" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D279" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E279" s="1" t="n">
         <v>38880</v>
@@ -5122,13 +5120,13 @@
         <v>15</v>
       </c>
       <c r="B280" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C280" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D280" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E280" s="1" t="n">
         <v>38880</v>
@@ -5139,13 +5137,13 @@
         <v>16</v>
       </c>
       <c r="B281" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C281" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D281" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E281" s="1" t="n">
         <v>38880</v>
@@ -5156,13 +5154,13 @@
         <v>5</v>
       </c>
       <c r="B282" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C282" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D282" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E282" s="1" t="n">
         <v>40320</v>
@@ -5170,16 +5168,16 @@
     </row>
     <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B283" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C283" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D283" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E283" s="1" t="n">
         <v>40320</v>
@@ -5190,13 +5188,13 @@
         <v>9</v>
       </c>
       <c r="B284" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C284" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D284" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E284" s="1" t="n">
         <v>40320</v>
@@ -5207,13 +5205,13 @@
         <v>10</v>
       </c>
       <c r="B285" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C285" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D285" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E285" s="1" t="n">
         <v>40320</v>
@@ -5224,13 +5222,13 @@
         <v>11</v>
       </c>
       <c r="B286" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C286" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D286" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E286" s="1" t="n">
         <v>40320</v>
@@ -5241,13 +5239,13 @@
         <v>12</v>
       </c>
       <c r="B287" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C287" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D287" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E287" s="1" t="n">
         <v>40320</v>
@@ -5258,13 +5256,13 @@
         <v>13</v>
       </c>
       <c r="B288" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C288" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D288" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E288" s="1" t="n">
         <v>40320</v>
@@ -5275,13 +5273,13 @@
         <v>14</v>
       </c>
       <c r="B289" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C289" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D289" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E289" s="1" t="n">
         <v>40320</v>
@@ -5292,13 +5290,13 @@
         <v>15</v>
       </c>
       <c r="B290" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C290" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D290" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E290" s="1" t="n">
         <v>40320</v>
@@ -5309,13 +5307,13 @@
         <v>16</v>
       </c>
       <c r="B291" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C291" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D291" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E291" s="1" t="n">
         <v>40320</v>
@@ -5326,13 +5324,13 @@
         <v>5</v>
       </c>
       <c r="B292" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C292" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D292" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E292" s="1" t="n">
         <v>41760</v>
@@ -5340,16 +5338,16 @@
     </row>
     <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B293" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C293" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D293" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E293" s="1" t="n">
         <v>41760</v>
@@ -5360,13 +5358,13 @@
         <v>9</v>
       </c>
       <c r="B294" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C294" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D294" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E294" s="1" t="n">
         <v>41760</v>
@@ -5377,13 +5375,13 @@
         <v>10</v>
       </c>
       <c r="B295" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C295" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D295" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E295" s="1" t="n">
         <v>41760</v>
@@ -5394,13 +5392,13 @@
         <v>11</v>
       </c>
       <c r="B296" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C296" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D296" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E296" s="1" t="n">
         <v>41760</v>
@@ -5411,13 +5409,13 @@
         <v>12</v>
       </c>
       <c r="B297" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C297" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D297" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E297" s="1" t="n">
         <v>41760</v>
@@ -5428,13 +5426,13 @@
         <v>13</v>
       </c>
       <c r="B298" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C298" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D298" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E298" s="1" t="n">
         <v>41760</v>
@@ -5445,13 +5443,13 @@
         <v>14</v>
       </c>
       <c r="B299" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C299" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D299" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E299" s="1" t="n">
         <v>41760</v>
@@ -5462,13 +5460,13 @@
         <v>15</v>
       </c>
       <c r="B300" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C300" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D300" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E300" s="1" t="n">
         <v>41760</v>
@@ -5479,13 +5477,13 @@
         <v>16</v>
       </c>
       <c r="B301" s="1" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="C301" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D301" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E301" s="1" t="n">
         <v>41760</v>

</xml_diff>